<commit_message>
Tambah Flight SMART ke tema SMART Patrol
Aplikasi log terbang drone DJI dan pengisian data SMART untuk foto drone,
dibuka di dalam dashboard. Spreadsheet awal ikut diperbarui.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193RVRbiyhb7LinqoiVWbAL
</commit_message>
<xml_diff>
--- a/data/Konten_Satu_Data_Tambora.xlsx
+++ b/data/Konten_Satu_Data_Tambora.xlsx
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="347">
   <si>
     <t xml:space="preserve">Panduan isi Satu Data Tambora</t>
   </si>
@@ -658,7 +658,7 @@
     <t xml:space="preserve">Spatial Monitoring and Reporting Tool</t>
   </si>
   <si>
-    <t xml:space="preserve">Temuan patroli dari seluruh resor: statistik, grafik per kategori, peta sebaran, dan pembuat laporan patroli.</t>
+    <t xml:space="preserve">Temuan patroli dari seluruh resor: statistik, grafik per kategori, peta sebaran, pembuat laporan patroli, dan data patroli drone.</t>
   </si>
   <si>
     <t xml:space="preserve">patroli</t>
@@ -977,6 +977,18 @@
   </si>
   <si>
     <t xml:space="preserve">kopluck8/SMART_Report_generator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight SMART</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://kopluck8.github.io/Flight_SMART/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arsip log terbang drone DJI (jalur GPX, KML, peta) dan pengisian data SMART untuk foto drone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kopluck8/Flight_SMART</t>
   </si>
   <si>
     <t xml:space="preserve">Rekap per kategori</t>
@@ -2206,7 +2218,7 @@
       </c>
       <c r="D47" s="8" t="n">
         <f aca="false">IF(Tema!$A3="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A3,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2358,7 +2370,7 @@
       </c>
       <c r="D58" s="10" t="n">
         <f aca="false">COUNTIFS(Item!$C$2:$C$400,"&lt;&gt;",Item!$J$2:$J$400,"&lt;&gt;tidak")</f>
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3765,45 +3777,47 @@
         <v>106</v>
       </c>
       <c r="B16" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="D16" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="13" t="s">
+      <c r="F16" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="G16" s="13"/>
+      <c r="H16" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
@@ -3812,24 +3826,24 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G18" s="13"/>
       <c r="H18" s="13"/>
@@ -3838,24 +3852,24 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
@@ -3869,19 +3883,19 @@
         <v>106</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
@@ -3895,19 +3909,19 @@
         <v>106</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D21" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="13"/>
@@ -3916,24 +3930,24 @@
         <v>105</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D22" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
@@ -3942,24 +3956,24 @@
         <v>105</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
@@ -3973,19 +3987,19 @@
         <v>106</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
@@ -3999,13 +4013,13 @@
         <v>106</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>244</v>
+        <v>220</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>245</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E25" s="13" t="s">
         <v>246</v>
@@ -4025,19 +4039,19 @@
         <v>106</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
@@ -4046,32 +4060,28 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>207</v>
+        <v>248</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G27" s="13"/>
-      <c r="H27" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
       <c r="J27" s="13" t="s">
         <v>105</v>
       </c>
@@ -4097,14 +4107,16 @@
       </c>
       <c r="G28" s="13"/>
       <c r="H28" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="I28" s="13"/>
+        <v>258</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J28" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
         <v>116</v>
       </c>
@@ -4112,20 +4124,20 @@
         <v>207</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G29" s="13"/>
       <c r="H29" s="13" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="I29" s="13"/>
       <c r="J29" s="13" t="s">
@@ -4137,13 +4149,13 @@
         <v>116</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>261</v>
+        <v>207</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>262</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E30" s="13" t="s">
         <v>263</v>
@@ -4152,7 +4164,9 @@
         <v>264</v>
       </c>
       <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
+      <c r="H30" s="13" t="s">
+        <v>258</v>
+      </c>
       <c r="I30" s="13"/>
       <c r="J30" s="13" t="s">
         <v>105</v>
@@ -4163,19 +4177,19 @@
         <v>116</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
@@ -4184,18 +4198,18 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C32" s="13" t="s">
         <v>269</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E32" s="13" t="s">
         <v>270</v>
@@ -4204,12 +4218,8 @@
         <v>271</v>
       </c>
       <c r="G32" s="13"/>
-      <c r="H32" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
       <c r="J32" s="13" t="s">
         <v>105</v>
       </c>
@@ -4219,7 +4229,7 @@
         <v>126</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C33" s="13" t="s">
         <v>273</v>
@@ -4237,17 +4247,19 @@
       <c r="H33" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="I33" s="13"/>
+      <c r="I33" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J33" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
         <v>126</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>277</v>
@@ -4263,53 +4275,53 @@
       </c>
       <c r="G34" s="13"/>
       <c r="H34" s="13" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="I34" s="13"/>
       <c r="J34" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
         <v>126</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G35" s="13"/>
       <c r="H35" s="13" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="I35" s="13"/>
       <c r="J35" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
         <v>126</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>244</v>
+        <v>272</v>
       </c>
       <c r="C36" s="13" t="s">
         <v>284</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E36" s="13" t="s">
         <v>285</v>
@@ -4318,7 +4330,9 @@
         <v>286</v>
       </c>
       <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
+      <c r="H36" s="13" t="s">
+        <v>287</v>
+      </c>
       <c r="I36" s="13"/>
       <c r="J36" s="13" t="s">
         <v>105</v>
@@ -4329,19 +4343,19 @@
         <v>126</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D37" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G37" s="13"/>
       <c r="H37" s="13"/>
@@ -4355,23 +4369,21 @@
         <v>126</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="G38" s="13" t="s">
         <v>293</v>
       </c>
+      <c r="G38" s="13"/>
       <c r="H38" s="13"/>
       <c r="I38" s="13"/>
       <c r="J38" s="13" t="s">
@@ -4380,28 +4392,28 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B39" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="C39" s="13" t="s">
         <v>294</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>295</v>
       </c>
       <c r="D39" s="13" t="s">
         <v>39</v>
       </c>
       <c r="E39" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="F39" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="F39" s="14" t="s">
+      <c r="G39" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="G39" s="13"/>
       <c r="H39" s="13"/>
-      <c r="I39" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="I39" s="13"/>
       <c r="J39" s="13" t="s">
         <v>105</v>
       </c>
@@ -4411,23 +4423,25 @@
         <v>135</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D40" s="13" t="s">
         <v>39</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G40" s="13"/>
       <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
+      <c r="I40" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J40" s="13" t="s">
         <v>105</v>
       </c>
@@ -4437,13 +4451,13 @@
         <v>135</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C41" s="13" t="s">
         <v>302</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="E41" s="13" t="s">
         <v>303</v>
@@ -4463,19 +4477,19 @@
         <v>135</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G42" s="13"/>
       <c r="H42" s="13"/>
@@ -4486,16 +4500,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>309</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E43" s="13" t="s">
         <v>310</v>
@@ -4503,13 +4517,9 @@
       <c r="F43" s="14" t="s">
         <v>311</v>
       </c>
-      <c r="G43" s="13" t="s">
-        <v>312</v>
-      </c>
+      <c r="G43" s="13"/>
       <c r="H43" s="13"/>
-      <c r="I43" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="I43" s="13"/>
       <c r="J43" s="13" t="s">
         <v>105</v>
       </c>
@@ -4519,23 +4529,27 @@
         <v>144</v>
       </c>
       <c r="B44" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="C44" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="C44" s="13" t="s">
+      <c r="D44" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E44" s="13" t="s">
         <v>314</v>
       </c>
-      <c r="D44" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" s="13" t="s">
+      <c r="F44" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="F44" s="14" t="s">
+      <c r="G44" s="13" t="s">
         <v>316</v>
       </c>
-      <c r="G44" s="13"/>
       <c r="H44" s="13"/>
-      <c r="I44" s="13"/>
+      <c r="I44" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J44" s="13" t="s">
         <v>105</v>
       </c>
@@ -4545,19 +4559,19 @@
         <v>144</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D45" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G45" s="13"/>
       <c r="H45" s="13"/>
@@ -4571,19 +4585,19 @@
         <v>144</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D46" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G46" s="13"/>
       <c r="H46" s="13"/>
@@ -4597,19 +4611,19 @@
         <v>144</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D47" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G47" s="13"/>
       <c r="H47" s="13"/>
@@ -4623,19 +4637,19 @@
         <v>144</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D48" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G48" s="13"/>
       <c r="H48" s="13"/>
@@ -4649,7 +4663,7 @@
         <v>144</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
       <c r="C49" s="13" t="s">
         <v>330</v>
@@ -4675,19 +4689,19 @@
         <v>144</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D50" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G50" s="13"/>
       <c r="H50" s="13"/>
@@ -4701,19 +4715,19 @@
         <v>144</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D51" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
@@ -4722,47 +4736,61 @@
         <v>105</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>207</v>
+        <v>333</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G52" s="13"/>
-      <c r="H52" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="I52" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="H52" s="13"/>
+      <c r="I52" s="13"/>
       <c r="J52" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13"/>
-      <c r="B53" s="13"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="14"/>
+    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>343</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>344</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>345</v>
+      </c>
       <c r="G53" s="13"/>
-      <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
-      <c r="J53" s="13"/>
+      <c r="H53" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="I53" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J53" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13"/>

</xml_diff>

<commit_message>
Rekap dan peta areal terbakar dari delineasi manual
Angka Kebakaran Hutan memakai delineasi manual dari Simulasi API Tambora (status/areal_terbakar.json):
luas di kawasan, per resor, dan areal baru per delineasi, dengan tautan ke peta. Bila belum ada
delineasi, tetap memakai estimasi Sentinel-2. Peta Sebaran Areal Terbakar diganti dengan
peta_terbakar.html yang diperbarui dari Google Drive.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193RVRbiyhb7LinqoiVWbAL
</commit_message>
<xml_diff>
--- a/data/Konten_Satu_Data_Tambora.xlsx
+++ b/data/Konten_Satu_Data_Tambora.xlsx
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="347">
   <si>
     <t xml:space="preserve">Panduan isi Satu Data Tambora</t>
   </si>
@@ -718,7 +718,7 @@
     <t xml:space="preserve">Pengendalian kebakaran hutan</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotspot harian, bekas terbakar dari citra satelit, peta kerawanan, rekap kejadian, dan pemodelan rambatan api.</t>
+    <t xml:space="preserve">Hotspot harian, delineasi areal terbakar tiap 5 hari, peta kerawanan, rekap kejadian, dan pemodelan rambatan api.</t>
   </si>
   <si>
     <t xml:space="preserve">api</t>
@@ -733,7 +733,7 @@
     <t xml:space="preserve">62% 50%</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotspot MODIS dan VIIRS; Bekas terbakar dari Sentinel-2; Simulasi rambatan api</t>
+    <t xml:space="preserve">Hotspot MODIS dan VIIRS; Delineasi areal terbakar tiap 5 hari; Simulasi rambatan api</t>
   </si>
   <si>
     <t xml:space="preserve">polhut</t>
@@ -1207,10 +1207,10 @@
     <t xml:space="preserve">Sebaran Areal Terbakar</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.google.com/maps/d/embed?mid=1mOK7vlcmfg8DN8Wr0OhR3Q_VK4ajzY4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peta sebaran areal bekas terbakar (burn area).</t>
+    <t xml:space="preserve">https://kopluck8.github.io/Simulasi-API-Tambora/peta_terbakar.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peta areal terbakar dari delineasi manual tiap 5 hari, dengan rekap per resor; diperbarui otomatis dari Google Drive.</t>
   </si>
   <si>
     <t xml:space="preserve">Rekap Kejadian Kebakaran Hutan</t>
@@ -4364,7 +4364,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
         <v>126</v>
       </c>
@@ -4384,7 +4384,9 @@
         <v>293</v>
       </c>
       <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
+      <c r="H38" s="13" t="s">
+        <v>280</v>
+      </c>
       <c r="I38" s="13"/>
       <c r="J38" s="13" t="s">
         <v>105</v>

</xml_diff>

<commit_message>
Tab Resor Pengelolaan: profil potensi dan ancaman tujuh resor 2026
- Halaman resor/: ikhtisar tujuh resor (peta batas 2026, peringkat ancaman
  dan potensi, beban kerja, perubahan batas), profil per resor, dan metode.
- Batas resor 2026 dari SHP kajian hanya dipakai di tab ini.
- tools/resor/olah_resor.py memadukan Laporan Kajian Wilayah Kerja Resor,
  data SMART Patrol, dan delineasi areal terbakar: ancaman dinilai dengan
  Miradi (lingkup x keparahan x ketakpulihan, kode IUCN-CMP, rangkuman
  3-5-7/2-prime), potensi dengan tiga fungsi kawasan konservasi.
- Workflow harian 07.40 WITA memperbarui data/resor/analisis.json dan
  peta.geojson.
- Hub: ubin Resor Pengelolaan, 9 kartu, angka langsung skor potensi,
  ikon pohon, link repo boleh memakai #bagian.
- Tempat foto per resor di data/resor/foto.json.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193RVRbiyhb7LinqoiVWbAL
</commit_message>
<xml_diff>
--- a/data/Konten_Satu_Data_Tambora.xlsx
+++ b/data/Konten_Satu_Data_Tambora.xlsx
@@ -70,7 +70,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Kode tema: huruf kecil tanpa spasi, contoh kawasan. Dipakai di alamat (#/kawasan) dan kolom tema di tab Item. Kode rbm, smart, dan karhut menampilkan angka langsung; jangan diganti.</t>
+          <t xml:space="preserve">Kode tema: huruf kecil tanpa spasi, contoh kawasan. Dipakai di alamat (#/kawasan) dan kolom tema di tab Item. Kode rbm, smart, karhut, dan resor menampilkan angka langsung; jangan diganti.</t>
         </r>
       </text>
     </comment>
@@ -118,7 +118,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Ikon pada ubin: gunung, patroli, resor, api, perisai, wisata, aset, peta, grafik, data, dokumen, folder, aplikasi, presentasi.</t>
+          <t xml:space="preserve">Ikon pada ubin: gunung, pohon, patroli, resor, api, perisai, wisata, aset, peta, grafik, data, dokumen, folder, aplikasi, presentasi.</t>
         </r>
       </text>
     </comment>
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="382">
   <si>
     <t xml:space="preserve">Panduan isi Satu Data Tambora</t>
   </si>
@@ -550,7 +550,7 @@
     <t xml:space="preserve">Angka langsung</t>
   </si>
   <si>
-    <t xml:space="preserve">Tema dengan id rbm, smart, dan karhut menampilkan angka terkini dari aplikasi Dashboard Capaian RBM, Dashboard SMART Patrol, dan Simulasi API Tambora. Jangan ganti ketiga id itu; judul, foto, dan isinya boleh diubah.</t>
+    <t xml:space="preserve">Tema dengan id rbm, smart, karhut, dan resor menampilkan angka terkini dari Dashboard Capaian RBM, Dashboard SMART Patrol, Simulasi API Tambora, dan analisis Resor Pengelolaan. Jangan ganti keempat id itu; judul, foto, dan isinya boleh diubah.</t>
   </si>
   <si>
     <t xml:space="preserve">Ringkasan (dihitung otomatis)</t>
@@ -649,6 +649,27 @@
     <t xml:space="preserve">ya</t>
   </si>
   <si>
+    <t xml:space="preserve">resor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Pengelolaan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tujuh resor hasil kajian 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profil potensi dan ancaman setiap resor pengelolaan: batas resor 2026, penilaian ancaman Miradi, temuan SMART Patrol, beban kerja, dan kebutuhan personel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pohon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#52c97c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 resor di 2 SPTN; Resor baru Doro Tabe; Potensi dan ancaman tiap resor</t>
+  </si>
+  <si>
     <t xml:space="preserve">smart</t>
   </si>
   <si>
@@ -691,9 +712,6 @@
     <t xml:space="preserve">Laporan kegiatan resor dan capaiannya terhadap rencana 2026, dihitung langsung dari laporan yang sudah diverifikasi.</t>
   </si>
   <si>
-    <t xml:space="preserve">resor</t>
-  </si>
-  <si>
     <t xml:space="preserve">#ffcf6e</t>
   </si>
   <si>
@@ -952,6 +970,96 @@
     <t xml:space="preserve">Peta desa binaan di sekitar kawasan.</t>
   </si>
   <si>
+    <t xml:space="preserve">Ikhtisar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profil Tujuh Resor Pengelolaan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peta batas resor 2026, peringkat ancaman dan potensi tiap resor, beban kerja, dan perubahan batas dari 6 menjadi 7 resor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metode Penilaian Potensi dan Ancaman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/metode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Penilaian ancaman Miradi (Conservation Standards), laju temuan SMART per 10 hari patroli, dan tiga fungsi kawasan konservasi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPTN Wilayah I Kore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Piong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/piong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Savana, pendakian berkendara, dan habitat Rusa timor. Desa binaan Piong dan Oi Saro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Oi Katupa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/oi-katupa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habitat Elang flores dan Rusa timor, madu hutan, dan sumber air. Desa binaan Oi Katupa, Kawinda Toi, dan Piong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Kawinda Toi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/kawinda-toi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wisata pendakian dan Air Terjun Oi Marai, madu hutan, dan sumber air. Desa binaan Kawinda Toi dan Kawinda Nae.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPTN Wilayah II Pekat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Doro Tabe (baru)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/doro-tabe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor baru 2026 dari pemekaran Doroncanga: savana dan fitur geologi. Desa binaan Tolokalo dan Soritatanga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Doroncanga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/doroncanga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanctuary Rusa Timor, savana, dan jalur pendakian berkendara. Desa binaan Soritatanga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Doropeti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/doropeti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Areal bernilai konservasi tinggi, habitat Elang flores, dan sumber air. Desa binaan Doropeti dan Soritatanga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resor Pancasila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resor/index.html#/pancasila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jalur pendakian ke puncak Tambora dan habitat Rusa timor. Desa binaan Tambora dan Kawinda Nae.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aplikasi</t>
   </si>
   <si>
@@ -1136,9 +1244,6 @@
   </si>
   <si>
     <t xml:space="preserve">Grafik beban kerja Balai TN Tambora.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resor Piong</t>
   </si>
   <si>
     <t xml:space="preserve">https://docs.google.com/spreadsheets/d/e/2CAIWO3emAV1x3glDUfwxF17DdMTFQ3Ir6qmjgL00uSfi205SDI1PS6XoWdV2LVBmWB5XiQoFZzOv80BSqRQ/gviz/chartiframe?autosize=true&amp;oid=915370174</t>
@@ -2210,99 +2315,99 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="7" t="str">
         <f aca="false">IF(Tema!$A3="","",Tema!$A3)</f>
-        <v>smart</v>
+        <v>resor</v>
       </c>
       <c r="C47" s="5" t="str">
         <f aca="false">IF(Tema!$A3="","",Tema!$B3)</f>
-        <v>SMART Patrol</v>
+        <v>Resor Pengelolaan</v>
       </c>
       <c r="D47" s="8" t="n">
         <f aca="false">IF(Tema!$A3="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A3,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="7" t="str">
         <f aca="false">IF(Tema!$A4="","",Tema!$A4)</f>
-        <v>rbm</v>
+        <v>smart</v>
       </c>
       <c r="C48" s="5" t="str">
         <f aca="false">IF(Tema!$A4="","",Tema!$B4)</f>
-        <v>Resort Based Management</v>
+        <v>SMART Patrol</v>
       </c>
       <c r="D48" s="8" t="n">
         <f aca="false">IF(Tema!$A4="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A4,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="7" t="str">
         <f aca="false">IF(Tema!$A5="","",Tema!$A5)</f>
-        <v>karhut</v>
+        <v>rbm</v>
       </c>
       <c r="C49" s="5" t="str">
         <f aca="false">IF(Tema!$A5="","",Tema!$B5)</f>
-        <v>Kebakaran Hutan</v>
+        <v>Resort Based Management</v>
       </c>
       <c r="D49" s="8" t="n">
         <f aca="false">IF(Tema!$A5="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A5,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="7" t="str">
         <f aca="false">IF(Tema!$A6="","",Tema!$A6)</f>
-        <v>polhut</v>
+        <v>karhut</v>
       </c>
       <c r="C50" s="5" t="str">
         <f aca="false">IF(Tema!$A6="","",Tema!$B6)</f>
-        <v>Perlindungan Kawasan</v>
+        <v>Kebakaran Hutan</v>
       </c>
       <c r="D50" s="8" t="n">
         <f aca="false">IF(Tema!$A6="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A6,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="7" t="str">
         <f aca="false">IF(Tema!$A7="","",Tema!$A7)</f>
-        <v>wisata</v>
+        <v>polhut</v>
       </c>
       <c r="C51" s="5" t="str">
         <f aca="false">IF(Tema!$A7="","",Tema!$B7)</f>
-        <v>Wisata &amp; Pelayanan</v>
+        <v>Perlindungan Kawasan</v>
       </c>
       <c r="D51" s="8" t="n">
         <f aca="false">IF(Tema!$A7="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A7,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="7" t="str">
         <f aca="false">IF(Tema!$A8="","",Tema!$A8)</f>
-        <v>bmn</v>
+        <v>wisata</v>
       </c>
       <c r="C52" s="5" t="str">
         <f aca="false">IF(Tema!$A8="","",Tema!$B8)</f>
-        <v>Aset BMN</v>
+        <v>Wisata &amp; Pelayanan</v>
       </c>
       <c r="D52" s="8" t="n">
         <f aca="false">IF(Tema!$A8="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A8,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="7" t="str">
         <f aca="false">IF(Tema!$A9="","",Tema!$A9)</f>
-        <v/>
+        <v>bmn</v>
       </c>
       <c r="C53" s="5" t="str">
         <f aca="false">IF(Tema!$A9="","",Tema!$B9)</f>
-        <v/>
-      </c>
-      <c r="D53" s="8" t="str">
+        <v>Aset BMN</v>
+      </c>
+      <c r="D53" s="8" t="n">
         <f aca="false">IF(Tema!$A9="","",COUNTIFS(Item!$A$2:$A$400,Tema!$A9,Item!$J$2:$J$400,"&lt;&gt;tidak",Item!$C$2:$C$400,"&lt;&gt;"))</f>
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2370,7 +2475,7 @@
       </c>
       <c r="D58" s="10" t="n">
         <f aca="false">COUNTIFS(Item!$C$2:$C$400,"&lt;&gt;",Item!$J$2:$J$400,"&lt;&gt;tidak")</f>
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2708,7 +2813,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
         <v>106</v>
       </c>
@@ -2727,17 +2832,11 @@
       <c r="F3" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="14" t="s">
         <v>112</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>115</v>
       </c>
       <c r="K3" s="13" t="s">
         <v>105</v>
@@ -2745,34 +2844,34 @@
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="E4" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="F4" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="G4" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="H4" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="I4" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="J4" s="14" t="s">
         <v>122</v>
-      </c>
-      <c r="H4" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="I4" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>125</v>
       </c>
       <c r="K4" s="13" t="s">
         <v>105</v>
@@ -2780,32 +2879,34 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="E5" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="G5" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="H5" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="I5" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="J5" s="14" t="s">
         <v>131</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H5" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="14" t="s">
-        <v>134</v>
       </c>
       <c r="K5" s="13" t="s">
         <v>105</v>
@@ -2813,32 +2914,32 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="E6" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="F6" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="G6" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="H6" s="13" t="s">
         <v>139</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>142</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="14" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="K6" s="13" t="s">
         <v>105</v>
@@ -2846,34 +2947,32 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="E7" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="F7" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="G7" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="F7" s="13" t="s">
+      <c r="H7" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="I7" s="13"/>
+      <c r="J7" s="14" t="s">
         <v>149</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="I7" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>152</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>105</v>
@@ -2881,45 +2980,67 @@
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="E8" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="F8" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="G8" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="H8" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="I8" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="J8" s="14" t="s">
         <v>158</v>
-      </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="14" t="s">
-        <v>159</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>164</v>
+      </c>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
       <c r="I9" s="13"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="13"/>
+      <c r="J9" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13"/>
@@ -3327,7 +3448,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation allowBlank="true" error="Pilih ikon dari daftar." errorStyle="warning" errorTitle="Ikon tidak dikenal" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E40" type="list">
-      <formula1>"gunung,patroli,resor,api,perisai,wisata,aset,peta,grafik,data,dokumen,folder,aplikasi,presentasi"</formula1>
+      <formula1>"gunung,pohon,patroli,resor,api,perisai,wisata,aset,peta,grafik,data,dokumen,folder,aplikasi,presentasi"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Isi tidak untuk menyembunyikan, atau kosongkan." errorStyle="warning" errorTitle="Isi ya atau tidak" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="K2:K40" type="list">
@@ -3368,10 +3489,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="C1" s="11" t="s">
         <v>54</v>
@@ -3380,19 +3501,19 @@
         <v>27</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="G1" s="12" t="s">
         <v>91</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="J1" s="12" t="s">
         <v>95</v>
@@ -3403,19 +3524,19 @@
         <v>96</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>44</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="G2" s="13"/>
       <c r="H2" s="13"/>
@@ -3431,19 +3552,19 @@
         <v>96</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="D3" s="13" t="s">
         <v>42</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -3457,19 +3578,19 @@
         <v>96</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
@@ -3483,19 +3604,19 @@
         <v>96</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="G5" s="13"/>
       <c r="H5" s="13"/>
@@ -3509,19 +3630,19 @@
         <v>96</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="G6" s="13"/>
       <c r="H6" s="13"/>
@@ -3535,19 +3656,19 @@
         <v>96</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -3561,22 +3682,22 @@
         <v>96</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>39</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
@@ -3589,19 +3710,19 @@
         <v>96</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>39</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
@@ -3615,19 +3736,19 @@
         <v>96</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
@@ -3641,19 +3762,19 @@
         <v>96</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>37</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
@@ -3667,19 +3788,19 @@
         <v>96</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
@@ -3693,19 +3814,19 @@
         <v>96</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
@@ -3714,28 +3835,28 @@
         <v>105</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="G14" s="13"/>
       <c r="H14" s="13" t="s">
-        <v>211</v>
+        <v>86</v>
       </c>
       <c r="I14" s="13" t="s">
         <v>105</v>
@@ -3749,23 +3870,23 @@
         <v>106</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="13" t="s">
-        <v>215</v>
+        <v>86</v>
       </c>
       <c r="I15" s="13"/>
       <c r="J15" s="13" t="s">
@@ -3777,23 +3898,23 @@
         <v>106</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="G16" s="13"/>
       <c r="H16" s="13" t="s">
-        <v>219</v>
+        <v>86</v>
       </c>
       <c r="I16" s="13"/>
       <c r="J16" s="13" t="s">
@@ -3808,25 +3929,27 @@
         <v>220</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
+      <c r="H17" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I17" s="13"/>
       <c r="J17" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
         <v>106</v>
       </c>
@@ -3834,19 +3957,21 @@
         <v>220</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
+      <c r="H18" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I18" s="13"/>
       <c r="J18" s="13" t="s">
         <v>105</v>
@@ -3857,100 +3982,108 @@
         <v>106</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
+      <c r="H19" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I19" s="13"/>
       <c r="J19" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
+      <c r="H20" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I20" s="13"/>
       <c r="J20" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
+      <c r="H21" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I21" s="13"/>
       <c r="J21" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
+      <c r="H22" s="13" t="s">
+        <v>86</v>
+      </c>
       <c r="I22" s="13"/>
       <c r="J22" s="13" t="s">
         <v>105</v>
@@ -3958,100 +4091,108 @@
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>220</v>
+        <v>243</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
+      <c r="H23" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J23" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>220</v>
+        <v>243</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
+      <c r="H24" s="13" t="s">
+        <v>251</v>
+      </c>
       <c r="I24" s="13"/>
       <c r="J24" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>220</v>
+        <v>243</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
+      <c r="H25" s="13" t="s">
+        <v>255</v>
+      </c>
       <c r="I25" s="13"/>
       <c r="J25" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
@@ -4062,22 +4203,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
@@ -4088,57 +4229,51 @@
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="G28" s="13"/>
-      <c r="H28" s="13" t="s">
-        <v>258</v>
-      </c>
-      <c r="I28" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
       <c r="J28" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="G29" s="13"/>
-      <c r="H29" s="13" t="s">
-        <v>258</v>
-      </c>
+      <c r="H29" s="13"/>
       <c r="I29" s="13"/>
       <c r="J29" s="13" t="s">
         <v>105</v>
@@ -4146,27 +4281,25 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="G30" s="13"/>
-      <c r="H30" s="13" t="s">
-        <v>258</v>
-      </c>
+      <c r="H30" s="13"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13" t="s">
         <v>105</v>
@@ -4174,22 +4307,22 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="D31" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
@@ -4198,24 +4331,24 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
@@ -4224,59 +4357,53 @@
         <v>105</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="G33" s="13"/>
-      <c r="H33" s="13" t="s">
-        <v>276</v>
-      </c>
-      <c r="I33" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
       <c r="J33" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="G34" s="13"/>
-      <c r="H34" s="13" t="s">
-        <v>280</v>
-      </c>
+      <c r="H34" s="13"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13" t="s">
         <v>105</v>
@@ -4284,108 +4411,108 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="G35" s="13"/>
-      <c r="H35" s="13" t="s">
-        <v>280</v>
-      </c>
+      <c r="H35" s="13"/>
       <c r="I35" s="13"/>
       <c r="J35" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="G36" s="13"/>
-      <c r="H36" s="13" t="s">
-        <v>287</v>
-      </c>
+      <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
+      <c r="H37" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="I37" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J37" s="13" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="G38" s="13"/>
       <c r="H38" s="13" t="s">
-        <v>280</v>
+        <v>294</v>
       </c>
       <c r="I38" s="13"/>
       <c r="J38" s="13" t="s">
@@ -4394,27 +4521,27 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C39" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>299</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13" t="s">
         <v>294</v>
       </c>
-      <c r="D39" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="F39" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>297</v>
-      </c>
-      <c r="H39" s="13"/>
       <c r="I39" s="13"/>
       <c r="J39" s="13" t="s">
         <v>105</v>
@@ -4422,50 +4549,48 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G40" s="13"/>
       <c r="H40" s="13"/>
-      <c r="I40" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="I40" s="13"/>
       <c r="J40" s="13" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>302</v>
+        <v>221</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
@@ -4474,53 +4599,59 @@
         <v>105</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
+      <c r="H42" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="I42" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J42" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
+      <c r="H43" s="13" t="s">
+        <v>315</v>
+      </c>
       <c r="I43" s="13"/>
       <c r="J43" s="13" t="s">
         <v>105</v>
@@ -4528,55 +4659,55 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B44" s="13" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F44" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="G44" s="13"/>
+      <c r="H44" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="G44" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="H44" s="13"/>
-      <c r="I44" s="13" t="s">
-        <v>105</v>
-      </c>
+      <c r="I44" s="13"/>
       <c r="J44" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G45" s="13"/>
-      <c r="H45" s="13"/>
+      <c r="H45" s="13" t="s">
+        <v>322</v>
+      </c>
       <c r="I45" s="13"/>
       <c r="J45" s="13" t="s">
         <v>105</v>
@@ -4584,22 +4715,22 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>317</v>
+        <v>284</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G46" s="13"/>
       <c r="H46" s="13"/>
@@ -4608,27 +4739,29 @@
         <v>105</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>317</v>
+        <v>284</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
+      <c r="H47" s="13" t="s">
+        <v>315</v>
+      </c>
       <c r="I47" s="13"/>
       <c r="J47" s="13" t="s">
         <v>105</v>
@@ -4636,24 +4769,26 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>317</v>
+        <v>284</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>329</v>
-      </c>
-      <c r="G48" s="13"/>
+        <v>331</v>
+      </c>
+      <c r="G48" s="13" t="s">
+        <v>332</v>
+      </c>
       <c r="H48" s="13"/>
       <c r="I48" s="13"/>
       <c r="J48" s="13" t="s">
@@ -4662,48 +4797,50 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
-      <c r="I49" s="13"/>
+      <c r="I49" s="13" t="s">
+        <v>105</v>
+      </c>
       <c r="J49" s="13" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B50" s="13" t="s">
         <v>333</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="G50" s="13"/>
       <c r="H50" s="13"/>
@@ -4714,22 +4851,22 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
@@ -4740,22 +4877,22 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="D52" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
@@ -4764,29 +4901,29 @@
         <v>105</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>207</v>
+        <v>347</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>345</v>
-      </c>
-      <c r="G53" s="13"/>
-      <c r="H53" s="13" t="s">
-        <v>346</v>
-      </c>
+        <v>350</v>
+      </c>
+      <c r="G53" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="H53" s="13"/>
       <c r="I53" s="13" t="s">
         <v>105</v>
       </c>
@@ -4795,112 +4932,242 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="13"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="14"/>
+      <c r="A54" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>353</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>354</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>355</v>
+      </c>
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
       <c r="I54" s="13"/>
-      <c r="J54" s="13"/>
+      <c r="J54" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="13"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="14"/>
+      <c r="A55" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>356</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>358</v>
+      </c>
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
       <c r="I55" s="13"/>
-      <c r="J55" s="13"/>
+      <c r="J55" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="13"/>
-      <c r="B56" s="13"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="14"/>
+      <c r="A56" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>359</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>361</v>
+      </c>
       <c r="G56" s="13"/>
       <c r="H56" s="13"/>
       <c r="I56" s="13"/>
-      <c r="J56" s="13"/>
+      <c r="J56" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="13"/>
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="14"/>
+      <c r="A57" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>362</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="F57" s="14" t="s">
+        <v>364</v>
+      </c>
       <c r="G57" s="13"/>
       <c r="H57" s="13"/>
       <c r="I57" s="13"/>
-      <c r="J57" s="13"/>
+      <c r="J57" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="13"/>
-      <c r="B58" s="13"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="14"/>
+      <c r="A58" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>352</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>366</v>
+      </c>
+      <c r="F58" s="14" t="s">
+        <v>367</v>
+      </c>
       <c r="G58" s="13"/>
       <c r="H58" s="13"/>
       <c r="I58" s="13"/>
-      <c r="J58" s="13"/>
+      <c r="J58" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="13"/>
-      <c r="B59" s="13"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="14"/>
+      <c r="A59" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>370</v>
+      </c>
+      <c r="F59" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="G59" s="13"/>
       <c r="H59" s="13"/>
       <c r="I59" s="13"/>
-      <c r="J59" s="13"/>
+      <c r="J59" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="13"/>
-      <c r="B60" s="13"/>
-      <c r="C60" s="13"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="13"/>
-      <c r="F60" s="14"/>
+      <c r="A60" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="F60" s="14" t="s">
+        <v>374</v>
+      </c>
       <c r="G60" s="13"/>
       <c r="H60" s="13"/>
       <c r="I60" s="13"/>
-      <c r="J60" s="13"/>
+      <c r="J60" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="13"/>
-      <c r="B61" s="13"/>
-      <c r="C61" s="13"/>
-      <c r="D61" s="13"/>
-      <c r="E61" s="13"/>
-      <c r="F61" s="14"/>
+      <c r="A61" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>376</v>
+      </c>
+      <c r="F61" s="14" t="s">
+        <v>377</v>
+      </c>
       <c r="G61" s="13"/>
       <c r="H61" s="13"/>
       <c r="I61" s="13"/>
-      <c r="J61" s="13"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="13"/>
-      <c r="B62" s="13"/>
-      <c r="C62" s="13"/>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13"/>
-      <c r="F62" s="14"/>
+      <c r="J61" s="13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="D62" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>379</v>
+      </c>
+      <c r="F62" s="14" t="s">
+        <v>380</v>
+      </c>
       <c r="G62" s="13"/>
-      <c r="H62" s="13"/>
-      <c r="I62" s="13"/>
-      <c r="J62" s="13"/>
+      <c r="H62" s="13" t="s">
+        <v>381</v>
+      </c>
+      <c r="I62" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J62" s="13" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="13"/>

</xml_diff>